<commit_message>
feat : modified coverage constraint to take into account abc class per outlet correctly, link channel type with channel id and divided by 14
</commit_message>
<xml_diff>
--- a/data/ExcelParameters/CoverageperABCperChannel.xlsx
+++ b/data/ExcelParameters/CoverageperABCperChannel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://loreal-my.sharepoint.com/personal/nils_levillain_loreal_com/Documents/Documents/Cline/nw-allocation-tool/data/ExcelParameters/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="8_{0AA7584F-D85B-436B-ABF0-9030EC79EE49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E00BC2CB-154D-453D-98C3-206EBDA195AD}"/>
+  <xr:revisionPtr revIDLastSave="21" documentId="8_{0AA7584F-D85B-436B-ABF0-9030EC79EE49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C2E68856-B46B-4448-B1B6-589994E5CA72}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{18B4B8A2-C4B4-4780-A18C-FFEAEF7D9308}"/>
   </bookViews>
@@ -38,9 +38,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="8">
   <si>
-    <t>Outlet</t>
-  </si>
-  <si>
     <t>A</t>
   </si>
   <si>
@@ -60,6 +57,9 @@
   </si>
   <si>
     <t>channel_id</t>
+  </si>
+  <si>
+    <t>outlet</t>
   </si>
 </sst>
 </file>
@@ -646,21 +646,21 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="5" t="s">
         <v>0</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>1</v>
       </c>
       <c r="C2" s="6">
         <v>28</v>
@@ -668,10 +668,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C3" s="6">
         <v>21</v>
@@ -679,10 +679,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C4" s="6">
         <v>14</v>
@@ -690,10 +690,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C5" s="6">
         <v>60</v>
@@ -701,10 +701,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C6" s="6">
         <v>45</v>
@@ -712,10 +712,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C7" s="6">
         <v>30</v>

</xml_diff>

<commit_message>
Memory bank updated ; addition of sellin file
</commit_message>
<xml_diff>
--- a/data/ExcelParameters/CoverageperABCperChannel.xlsx
+++ b/data/ExcelParameters/CoverageperABCperChannel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://loreal-my.sharepoint.com/personal/nils_levillain_loreal_com/Documents/Documents/Cline/nw-allocation-tool/data/ExcelParameters/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="21" documentId="8_{0AA7584F-D85B-436B-ABF0-9030EC79EE49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C2E68856-B46B-4448-B1B6-589994E5CA72}"/>
+  <xr:revisionPtr revIDLastSave="34" documentId="8_{0AA7584F-D85B-436B-ABF0-9030EC79EE49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{38E7CEBB-AC24-4122-A1FF-CD3A6A0BF703}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{18B4B8A2-C4B4-4780-A18C-FFEAEF7D9308}"/>
   </bookViews>
@@ -663,7 +663,7 @@
         <v>0</v>
       </c>
       <c r="C2" s="6">
-        <v>28</v>
+        <v>180</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -674,7 +674,7 @@
         <v>1</v>
       </c>
       <c r="C3" s="6">
-        <v>21</v>
+        <v>170</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
@@ -685,7 +685,7 @@
         <v>2</v>
       </c>
       <c r="C4" s="6">
-        <v>14</v>
+        <v>160</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">

</xml_diff>